<commit_message>
Added some experimental data from Fugaku machine on BLUF
</commit_message>
<xml_diff>
--- a/experiments/segmented-mem/fugaku/large-input-experiments-data.xlsx
+++ b/experiments/segmented-mem/fugaku/large-input-experiments-data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Programming\HighP5\experiments\segmented-mem\fugaku\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D47CD2AD-CD3F-47C8-9B16-729DE3416956}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{27701CDB-2E13-4A26-8B02-CF2B485CC12F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="HighP5-Bluf" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="10">
   <si>
     <t>Memory</t>
   </si>
@@ -67,6 +67,9 @@
   <si>
     <t>100 Nodes 8 MPI Processes Per Node. A 51200 by 51200 Square Matrix that is 90% Sparse and 51200 gradient descend iterations.</t>
   </si>
+  <si>
+    <t>200 Nodes 32 MPI Process Per Node for 51200 by 51200 Matrix</t>
+  </si>
 </sst>
 </file>
 
@@ -89,7 +92,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -105,6 +108,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="2" tint="-9.9978637043366805E-2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.79998168889431442"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -136,11 +145,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -788,7 +801,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{84CD9A06-15EE-46AA-8E1C-8081451551F4}">
-  <dimension ref="A1:H14"/>
+  <dimension ref="A1:H28"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="12.77734375" customWidth="1"/>
@@ -810,6 +823,10 @@
       <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
+      <c r="E1" s="4"/>
+      <c r="F1" s="4"/>
+      <c r="G1" s="4"/>
+      <c r="H1" s="4"/>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A2">
@@ -824,6 +841,10 @@
       <c r="D2">
         <v>1627.44</v>
       </c>
+      <c r="E2" s="4"/>
+      <c r="F2" s="4"/>
+      <c r="G2" s="4"/>
+      <c r="H2" s="4"/>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A3">
@@ -838,6 +859,10 @@
       <c r="D3">
         <v>2078.81</v>
       </c>
+      <c r="E3" s="4"/>
+      <c r="F3" s="4"/>
+      <c r="G3" s="4"/>
+      <c r="H3" s="4"/>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A4">
@@ -852,6 +877,10 @@
       <c r="D4">
         <v>2090.36</v>
       </c>
+      <c r="E4" s="4"/>
+      <c r="F4" s="4"/>
+      <c r="G4" s="4"/>
+      <c r="H4" s="4"/>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A5">
@@ -866,11 +895,12 @@
       <c r="D5">
         <v>1704.93</v>
       </c>
-      <c r="F5" s="3" t="s">
+      <c r="E5" s="4"/>
+      <c r="F5" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="G5" s="3"/>
-      <c r="H5" s="3"/>
+      <c r="G5" s="5"/>
+      <c r="H5" s="5"/>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A6">
@@ -885,9 +915,10 @@
       <c r="D6">
         <v>1864.52</v>
       </c>
-      <c r="F6" s="3"/>
-      <c r="G6" s="3"/>
-      <c r="H6" s="3"/>
+      <c r="E6" s="4"/>
+      <c r="F6" s="5"/>
+      <c r="G6" s="5"/>
+      <c r="H6" s="5"/>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A7">
@@ -902,9 +933,10 @@
       <c r="D7">
         <v>2368.92</v>
       </c>
-      <c r="F7" s="3"/>
-      <c r="G7" s="3"/>
-      <c r="H7" s="3"/>
+      <c r="E7" s="4"/>
+      <c r="F7" s="5"/>
+      <c r="G7" s="5"/>
+      <c r="H7" s="5"/>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A8">
@@ -919,9 +951,10 @@
       <c r="D8">
         <v>1861.48</v>
       </c>
-      <c r="F8" s="3"/>
-      <c r="G8" s="3"/>
-      <c r="H8" s="3"/>
+      <c r="E8" s="4"/>
+      <c r="F8" s="5"/>
+      <c r="G8" s="5"/>
+      <c r="H8" s="5"/>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A9">
@@ -936,9 +969,10 @@
       <c r="D9">
         <v>2189.15</v>
       </c>
-      <c r="F9" s="3"/>
-      <c r="G9" s="3"/>
-      <c r="H9" s="3"/>
+      <c r="E9" s="4"/>
+      <c r="F9" s="5"/>
+      <c r="G9" s="5"/>
+      <c r="H9" s="5"/>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A10">
@@ -953,9 +987,10 @@
       <c r="D10">
         <v>2357.83</v>
       </c>
-      <c r="F10" s="3"/>
-      <c r="G10" s="3"/>
-      <c r="H10" s="3"/>
+      <c r="E10" s="4"/>
+      <c r="F10" s="5"/>
+      <c r="G10" s="5"/>
+      <c r="H10" s="5"/>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A11">
@@ -970,9 +1005,10 @@
       <c r="D11">
         <v>1925.3</v>
       </c>
-      <c r="F11" s="3"/>
-      <c r="G11" s="3"/>
-      <c r="H11" s="3"/>
+      <c r="E11" s="4"/>
+      <c r="F11" s="5"/>
+      <c r="G11" s="5"/>
+      <c r="H11" s="5"/>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A12">
@@ -987,6 +1023,10 @@
       <c r="D12">
         <v>1842.54</v>
       </c>
+      <c r="E12" s="4"/>
+      <c r="F12" s="4"/>
+      <c r="G12" s="4"/>
+      <c r="H12" s="4"/>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A13">
@@ -1001,6 +1041,10 @@
       <c r="D13">
         <v>2073.11</v>
       </c>
+      <c r="E13" s="4"/>
+      <c r="F13" s="4"/>
+      <c r="G13" s="4"/>
+      <c r="H13" s="4"/>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A14" s="1">
@@ -1019,10 +1063,219 @@
         <f t="shared" si="0"/>
         <v>1998.699166666667</v>
       </c>
+      <c r="E14" s="4"/>
+      <c r="F14" s="4"/>
+      <c r="G14" s="4"/>
+      <c r="H14" s="4"/>
+    </row>
+    <row r="18" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A18" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B18" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C18" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D18" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E18" s="4"/>
+      <c r="F18" s="4"/>
+      <c r="G18" s="4"/>
+      <c r="H18" s="4"/>
+    </row>
+    <row r="19" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A19">
+        <v>1447.64</v>
+      </c>
+      <c r="B19">
+        <v>449.68</v>
+      </c>
+      <c r="C19">
+        <v>1218.73</v>
+      </c>
+      <c r="D19">
+        <v>3116.05</v>
+      </c>
+      <c r="E19" s="4"/>
+      <c r="F19" s="4"/>
+      <c r="G19" s="4"/>
+      <c r="H19" s="4"/>
+    </row>
+    <row r="20" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A20">
+        <v>1588.82</v>
+      </c>
+      <c r="B20">
+        <v>480.904</v>
+      </c>
+      <c r="C20">
+        <v>1217.48</v>
+      </c>
+      <c r="D20">
+        <v>3287.2</v>
+      </c>
+      <c r="E20" s="4"/>
+      <c r="F20" s="4"/>
+      <c r="G20" s="4"/>
+      <c r="H20" s="4"/>
+    </row>
+    <row r="21" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A21">
+        <v>656.37800000000004</v>
+      </c>
+      <c r="B21">
+        <v>536.24699999999996</v>
+      </c>
+      <c r="C21">
+        <v>1217.8</v>
+      </c>
+      <c r="D21">
+        <v>2410.4299999999998</v>
+      </c>
+      <c r="E21" s="4"/>
+      <c r="F21" s="4"/>
+      <c r="G21" s="4"/>
+      <c r="H21" s="4"/>
+    </row>
+    <row r="22" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A22">
+        <v>1488.66</v>
+      </c>
+      <c r="B22">
+        <v>479.952</v>
+      </c>
+      <c r="C22">
+        <v>1218.04</v>
+      </c>
+      <c r="D22">
+        <v>3186.65</v>
+      </c>
+      <c r="E22" s="4"/>
+      <c r="F22" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="G22" s="5"/>
+      <c r="H22" s="5"/>
+    </row>
+    <row r="23" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A23">
+        <v>1021.88</v>
+      </c>
+      <c r="B23">
+        <v>571.93499999999995</v>
+      </c>
+      <c r="C23">
+        <v>1217.04</v>
+      </c>
+      <c r="D23">
+        <v>2810.85</v>
+      </c>
+      <c r="E23" s="4"/>
+      <c r="F23" s="5"/>
+      <c r="G23" s="5"/>
+      <c r="H23" s="5"/>
+    </row>
+    <row r="24" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A24">
+        <v>809.02099999999996</v>
+      </c>
+      <c r="B24">
+        <v>514.68499999999995</v>
+      </c>
+      <c r="C24">
+        <v>1217.78</v>
+      </c>
+      <c r="D24">
+        <v>2541.4899999999998</v>
+      </c>
+      <c r="E24" s="4"/>
+      <c r="F24" s="5"/>
+      <c r="G24" s="5"/>
+      <c r="H24" s="5"/>
+    </row>
+    <row r="25" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A25">
+        <v>798.60400000000004</v>
+      </c>
+      <c r="B25">
+        <v>461.41199999999998</v>
+      </c>
+      <c r="C25">
+        <v>1216.95</v>
+      </c>
+      <c r="D25">
+        <v>2476.96</v>
+      </c>
+      <c r="E25" s="4"/>
+      <c r="F25" s="5"/>
+      <c r="G25" s="5"/>
+      <c r="H25" s="5"/>
+    </row>
+    <row r="26" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A26">
+        <v>1111.05</v>
+      </c>
+      <c r="B26">
+        <v>471.07499999999999</v>
+      </c>
+      <c r="C26">
+        <v>1217.3</v>
+      </c>
+      <c r="D26">
+        <v>2799.43</v>
+      </c>
+      <c r="E26" s="4"/>
+      <c r="F26" s="5"/>
+      <c r="G26" s="5"/>
+      <c r="H26" s="5"/>
+    </row>
+    <row r="27" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A27">
+        <v>788.68299999999999</v>
+      </c>
+      <c r="B27">
+        <v>504.75799999999998</v>
+      </c>
+      <c r="C27">
+        <v>2082.98</v>
+      </c>
+      <c r="D27">
+        <v>3376.42</v>
+      </c>
+      <c r="E27" s="4"/>
+      <c r="F27" s="5"/>
+      <c r="G27" s="5"/>
+      <c r="H27" s="5"/>
+    </row>
+    <row r="28" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A28" s="1">
+        <f>AVERAGE(A19:A27)</f>
+        <v>1078.9706666666668</v>
+      </c>
+      <c r="B28" s="1">
+        <f>AVERAGE(B19:B27)</f>
+        <v>496.73866666666657</v>
+      </c>
+      <c r="C28" s="1">
+        <f>AVERAGE(C19:C27)</f>
+        <v>1313.7888888888888</v>
+      </c>
+      <c r="D28" s="1">
+        <f>AVERAGE(D19:D27)</f>
+        <v>2889.4977777777772</v>
+      </c>
+      <c r="E28" s="4"/>
+      <c r="F28" s="4"/>
+      <c r="G28" s="4"/>
+      <c r="H28" s="4"/>
     </row>
   </sheetData>
-  <mergeCells count="1">
+  <mergeCells count="2">
     <mergeCell ref="F5:H11"/>
+    <mergeCell ref="F22:H27"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>

</xml_diff>